<commit_message>
Rebuild compiled employee list with photos embedded per employee (blank space where none)
</commit_message>
<xml_diff>
--- a/Compiled_Employee_List.xlsx
+++ b/Compiled_Employee_List.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,10 +28,20 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -40,7 +50,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE3F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4C7E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,35 +84,50 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D4DC"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D4DC"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D4DC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D4DC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -158,6 +203,1011 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="647700" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="666750" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="933450" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="504825" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="561975" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="504825" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="733425" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="438150" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="438150" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="438150" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="704850" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="600075" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="628650" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="581025" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="695325" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="590550" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="581025" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="590550" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="438150" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="647700" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="781050" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="638175" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -449,7 +1499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -462,1413 +1512,1432 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>COMPILED EMPLOYEE LIST  —  ALL BRANDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Total: 44 employees across 7 brands   |   Brands: Bigg Bear, B2B, Eggspert, OG Pizza, Koby's, The Chatpata Affair, The Momo Box</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>S. No.</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Employee ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Contact Number</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Aadhaar No</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>PAN No</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+    <row r="4" ht="69.5" customHeight="1">
+      <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Bigg Bear</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>AOT0001</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Saurabh Pandey</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>7289913393</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="69.5" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Bigg Bear</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>AOT0002</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Prakash Kumar</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>9310199259</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="69.5" customHeight="1">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Bigg Bear</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>AOT0003</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Kailash Joshi</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>8954742562</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7" ht="69.5" customHeight="1">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Bigg Bear</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>AOT0004</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Vijay Singh</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>6350367901</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="69.5" customHeight="1">
+      <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Bigg Bear</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>AOT0005</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Dipak</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>8318752699</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9" ht="69.5" customHeight="1">
+      <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Bigg Bear</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>AOT0006</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Aneesh Kumar</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>6306177706</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="69.5" customHeight="1">
+      <c r="A10" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Chirag Sharma</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>7906807310</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>4261 5309 3429</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="G10" s="7" t="inlineStr"/>
+      <c r="H10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="69.5" customHeight="1">
+      <c r="A11" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Vishwa Vardhan</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>8126677368</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>6202 8944 8807</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>CPHPC3097K</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="H11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="69.5" customHeight="1">
+      <c r="A12" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Mahipal</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>8800731018</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>7703 1482 9611</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>IHBPS7614</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="H12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="69.5" customHeight="1">
+      <c r="A13" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Vijay Negi</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>7088257652</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>4236 4897 7025</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="69.5" customHeight="1">
+      <c r="A14" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr"/>
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Aman</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>7678308172</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>4997 4265 3338</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="G14" s="7" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="69.5" customHeight="1">
+      <c r="A15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>kamal</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>9368096742</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>2632 8219 2034</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="69.5" customHeight="1">
+      <c r="A16" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr"/>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Naveen</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>9354806098</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>3267 6953 2169</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>GFCPK8064P</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="H16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="69.5" customHeight="1">
+      <c r="A17" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr"/>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Gaurav kumar</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>7060260302</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>4843 9988 6438</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>IZHPK0472E</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="H17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="69.5" customHeight="1">
+      <c r="A18" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr"/>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Karan kumar</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>9548076814</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>9510 6354 3190</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>GEMPM6841D</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="H18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="69.5" customHeight="1">
+      <c r="A19" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr"/>
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>Aakash Maurya</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>6398813187</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>7764 1385 4535</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>HAFPM4523J</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="H19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20" ht="69.5" customHeight="1">
+      <c r="A20" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr"/>
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>Ashish</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>9389789418</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>5161 5249 6798</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="G20" s="7" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="69.5" customHeight="1">
+      <c r="A21" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr"/>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Saurabh singh</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>7453819039</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>9272 5246 6390</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>PJJPS4565K</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="H21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="69.5" customHeight="1">
+      <c r="A22" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr"/>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Sundaram</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>9354806098</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>9454 7330 3411</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="G22" s="7" t="inlineStr"/>
+      <c r="H22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23" ht="69.5" customHeight="1">
+      <c r="A23" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr"/>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Arpit</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>7818004458</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>2849 4261 4953</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="G23" s="7" t="inlineStr"/>
+      <c r="H23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24" ht="69.5" customHeight="1">
+      <c r="A24" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr"/>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Deepak</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>9123470127</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>9257 1112 2002</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="G24" s="7" t="inlineStr"/>
+      <c r="H24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25" ht="69.5" customHeight="1">
+      <c r="A25" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Eggspert</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>NF0044</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>MUKUL</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>8588812227</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>8368 7527 5720</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>BJNPC0448M</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="H25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="69.5" customHeight="1">
+      <c r="A26" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Eggspert</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>AMIT</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>921330065</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>3257 5839 4988</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>CFZPC8635R</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="H26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27" ht="69.5" customHeight="1">
+      <c r="A27" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Eggspert</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>NF0130</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>DEEPKA</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>8287918813</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>8419 2625 4489</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>PHBPS2693C</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="H27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28" ht="69.5" customHeight="1">
+      <c r="A28" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Eggspert</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>NF0163</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>AJAY KUMAR</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>9990601136</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>4843 4760 5521</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>DNVPK7397M</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="H28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29" ht="69.5" customHeight="1">
+      <c r="A29" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>OG Pizza</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Saurabh Kumar</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>8102449112</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>3499 8671 8301</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="G29" s="7" t="inlineStr"/>
+      <c r="H29" s="7" t="inlineStr"/>
+    </row>
+    <row r="30" ht="69.5" customHeight="1">
+      <c r="A30" s="7" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>OG Pizza</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>002</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Gulshan Kumar</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>8076956211</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F30" s="8" t="inlineStr">
         <is>
           <t>6736 4525 9807</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="G30" s="7" t="inlineStr"/>
+      <c r="H30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31" ht="69.5" customHeight="1">
+      <c r="A31" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>OG Pizza</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>003</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>Satish</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>7078868439</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>5915 8835 1834</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="G31" s="7" t="inlineStr"/>
+      <c r="H31" s="7" t="inlineStr"/>
+    </row>
+    <row r="32" ht="69.5" customHeight="1">
+      <c r="A32" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Jitesh Kumar</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>9528957596</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>4820 6250 7730</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>PCNPK4619B</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="H32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33" ht="69.5" customHeight="1">
+      <c r="A33" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Komal</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>7011019098</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>7418 7170 7505</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>HCTPK3945Q</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="H33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34" ht="69.5" customHeight="1">
+      <c r="A34" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr"/>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Aditya</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>8279738969</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>7270 7424 4245</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>LCGPK1340E</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="H34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35" ht="69.5" customHeight="1">
+      <c r="A35" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Sahil</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>9971885713</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>3032 8966 0747</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>JXCPS4076J</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="H35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36" ht="69.5" customHeight="1">
+      <c r="A36" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>Yash Kumar</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>8375866689</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>3386 9082 6639</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>JSXPK4294J</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="H36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37" ht="69.5" customHeight="1">
+      <c r="A37" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Ishan Polusta</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>8394077593</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>5469 9556 6103</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>FRCPP1227G</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="H37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38" ht="69.5" customHeight="1">
+      <c r="A38" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr"/>
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>Shubham biswas</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>8810337785</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>3827 4390 0256</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>DPWPB8183P</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="H38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="69.5" customHeight="1">
+      <c r="A39" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Damodar Jha</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>8368399533</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>9769 8073 4887</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>AUEPJ1375R</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="H39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40" ht="69.5" customHeight="1">
+      <c r="A40" s="7" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>The Chatpata Affair</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>204</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>SANTOSH KUMAR</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E40" s="8" t="inlineStr">
         <is>
           <t>9305946728</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F40" s="8" t="inlineStr">
         <is>
           <t>6158 6990 5833</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="G40" s="7" t="inlineStr"/>
+      <c r="H40" s="7" t="inlineStr"/>
+    </row>
+    <row r="41" ht="69.5" customHeight="1">
+      <c r="A41" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>The Chatpata Affair</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>205</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D41" s="9" t="inlineStr">
         <is>
           <t>GAURAV ARYA</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t>8006058432</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>2354 4261 0569</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="G41" s="7" t="inlineStr"/>
+      <c r="H41" s="7" t="inlineStr"/>
+    </row>
+    <row r="42" ht="69.5" customHeight="1">
+      <c r="A42" s="7" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>The Chatpata Affair</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>207</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D42" s="9" t="inlineStr">
         <is>
           <t>NARENDRA KUMAR ARYA</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E42" s="8" t="inlineStr">
         <is>
           <t>9690999212</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t>2461 0635 8804</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="G42" s="7" t="inlineStr"/>
+      <c r="H42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43" ht="69.5" customHeight="1">
+      <c r="A43" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>The Chatpata Affair</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>206</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D43" s="9" t="inlineStr">
         <is>
           <t>SAHIL</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="8" t="inlineStr">
         <is>
           <t>7070621218</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="F43" s="8" t="inlineStr"/>
+      <c r="G43" s="7" t="inlineStr">
         <is>
           <t>GHCPK3642K</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="H43" s="7" t="inlineStr"/>
+    </row>
+    <row r="44" ht="64" customHeight="1">
+      <c r="A44" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>The Momo Box</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>Himanshu</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>8130665709</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>5482 8020 7052</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>BQZYP2738R</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="H44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45" ht="64" customHeight="1">
+      <c r="A45" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>The Momo Box</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Puran</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>8796947759</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t>6130 7492 0781</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>DELPC3338P</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="H45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="64" customHeight="1">
+      <c r="A46" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>The Momo Box</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>Kalash</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>8979575384</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>5017 1971 5384</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>DIRPK0597Q</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="H46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47" ht="64" customHeight="1">
+      <c r="A47" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>The Momo Box</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Sonu Yadav</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>7673822529</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>5407 1727 6431</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>OSJPK1327K</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Burrito Bros brand (4 employees) with photos to compiled list
</commit_message>
<xml_diff>
--- a/Compiled_Employee_List.xlsx
+++ b/Compiled_Employee_List.xlsx
@@ -228,6 +228,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -253,6 +256,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -278,6 +284,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -303,6 +312,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -328,6 +340,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -353,6 +368,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -378,6 +396,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -403,6 +424,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -428,6 +452,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -453,6 +480,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -478,6 +508,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -503,6 +536,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -528,6 +564,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -553,6 +592,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -578,6 +620,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -603,6 +648,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -628,6 +676,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -653,6 +704,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -678,6 +732,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -703,6 +760,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -728,6 +788,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -753,6 +816,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -778,6 +844,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -803,6 +872,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -828,6 +900,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -853,6 +928,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -878,6 +956,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -903,6 +984,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -928,6 +1012,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -953,6 +1040,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -978,6 +1068,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1003,6 +1096,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1028,6 +1124,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1053,6 +1152,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1078,6 +1180,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1103,6 +1208,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1128,6 +1236,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1153,6 +1264,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1178,6 +1292,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1197,6 +1314,109 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="876300" cy="1562100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1257300" cy="1562100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1171575" cy="1562100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1171575" cy="1562100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1499,7 +1719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1522,7 +1742,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total: 44 employees across 7 brands   |   Brands: Bigg Bear, B2B, Eggspert, OG Pizza, Koby's, The Chatpata Affair, The Momo Box</t>
+          <t>Total: 48 employees across 8 brands   |   Brands: Bigg Bear, B2B, Eggspert, OG Pizza, Koby's, The Chatpata Affair, The Momo Box, Burrito Bros</t>
         </is>
       </c>
     </row>
@@ -2931,6 +3151,150 @@
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48" ht="69.5" customHeight="1">
+      <c r="A48" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Burrito Bros</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>BB01</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>JATIN JHAWAR</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>6202282230</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>9588 8197 0484</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>CJFPJ9997M</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="n"/>
+    </row>
+    <row r="49" ht="69.5" customHeight="1">
+      <c r="A49" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Burrito Bros</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>BB02</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>KESHAV JHAWAR</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>7762040281</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>6383 4826 6615</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>BSXPJ2392A</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="n"/>
+    </row>
+    <row r="50" ht="69.5" customHeight="1">
+      <c r="A50" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Burrito Bros</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>BB03</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>MILAN SUBEDI</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>7770872441</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>9333 0098 4316</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>SHTPS2995L</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="n"/>
+    </row>
+    <row r="51" ht="69.5" customHeight="1">
+      <c r="A51" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Burrito Bros</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>BB04</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>MANOJ</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>7668864718</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>3821 2210 4800</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>HKMPM9433A</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>